<commit_message>
Re-check the question bank against the 28 new corpus pages
</commit_message>
<xml_diff>
--- a/eval/question_bank.xlsx
+++ b/eval/question_bank.xlsx
@@ -1253,37 +1253,37 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>함정-무근거</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>건축학전공은 졸업학점이 몇이야?</t>
+          <t>학사경고 받으면 다음 학기에 수강신청할 수 있는 학점이 줄어들어?</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>How many credits does the Architecture major require for graduation?</t>
+          <t>If I get an academic warning, will my credit limit for next semester be reduced?</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>158학점 (2016학번부터). 그 전 학번은 160·164</t>
+          <t>(자료에 없음. 학칙에는 학사경고 기준만 있음 → 학과 교학팀·교무팀 안내가 정답)</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>아주대학교 학칙, 학사지원 졸업 안내</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>제50조(학사과정의 졸업요건) ① · https://rules.ajou.ac.kr/IRS/rule/detail/594</t>
+          <t>(학칙 제47조는 학사경고 기준만 규정)</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>158이면 정답. 학번 차이를 언급해도 정답. 160·164를 단정하면 오답</t>
+          <t>수강 학점이 줄어든다거나 몇 학점으로 제한된다고 지어내면 오답. 학사경고 기준만 안내하고 수강 제한은 확인하라고 하면 정답</t>
         </is>
       </c>
       <c r="J13" s="10" t="n"/>
@@ -1291,7 +1291,7 @@
       <c r="L13" s="11" t="n"/>
       <c r="M13" s="11" t="inlineStr">
         <is>
-          <t>구간 A</t>
+          <t>구간 C · 10/27 재점검: 기존 '건축학전공 졸업학점'(9·18번과 겹침)을 새 함정으로 교체</t>
         </is>
       </c>
     </row>
@@ -1697,12 +1697,12 @@
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>학사지원 졸업 안내</t>
+          <t>아주대학교 졸업 안내</t>
         </is>
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>연도별 졸업요건 · https://www.ajou.ac.kr/kr/bachelor/regs-graduation.do</t>
+          <t>졸업요건 · https://www.ajou.ac.kr/kr/bachelor/regs-graduation.do</t>
         </is>
       </c>
       <c r="I21" s="11" t="inlineStr">
@@ -1715,7 +1715,7 @@
       <c r="L21" s="11" t="n"/>
       <c r="M21" s="11" t="inlineStr">
         <is>
-          <t>구간 A · 근거 페이지가 DB에 들어오기 전에는 오답 예상 — RAG 전후 비교 사례</t>
+          <t>구간 A · 10/25 이전 DB에는 근거 없음 → RAG 전후 비교 사례</t>
         </is>
       </c>
     </row>
@@ -1919,7 +1919,7 @@
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>대학원 규정을 학부에 적용하거나 상한을 지어내면 오답</t>
+          <t>대학원 규정(F 과목만 재수강)이나 학위취득유예생 재수강 규칙을 일반 학부 재수강 규칙으로 쓰거나, 상한을 지어내면 오답</t>
         </is>
       </c>
       <c r="J25" s="10" t="n"/>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>함정-무근거</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -1957,22 +1957,22 @@
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>(학부 수강신청 학점은 학사운영규칙 소관, 자료에 없음 → 안내가 정답)</t>
+          <t>학번·학과·성적에 따라 다름: 2004학번 이후 19학점(누계평점 3.75 이상 22학점), 소프트웨어학과·국방디지털융합학과는 21학점(3.75 이상 24학점), 2003학번까지 21학점(24학점)</t>
         </is>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아주대학교 수강신청 안내</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>(학칙 제46조①③)</t>
+          <t>수강신청학점 · https://www.ajou.ac.kr/kr/bachelor/enrolment.do</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>대학원의 12학점을 학부로 말하면 오답</t>
+          <t>학번·학과·평점에 따라 다르다는 점과 맞는 기준을 말하면 정답. 대학원 12학점이나 다른 값을 단정하면 오답</t>
         </is>
       </c>
       <c r="J26" s="10" t="n"/>
@@ -1980,7 +1980,7 @@
       <c r="L26" s="11" t="n"/>
       <c r="M26" s="11" t="inlineStr">
         <is>
-          <t>구간 C</t>
+          <t>구간 B · 10/27 재점검: 수강신청 안내 페이지 추가로 근거 생김 (함정 → B)</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>함정-무근거</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
@@ -2010,22 +2010,22 @@
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>(세부 기준은 학사운영규칙 소관, 자료에 없음 → 안내가 정답)</t>
+          <t>학번에 따라 다름: 2004~2013학번은 누계평점 2.50 이상(학기당 평균 14학점 이수), 2014~2024학번은 1학년 권장교육과정 이수가 원칙, 2025학번 이후는 전공과목 이수 요건. 최근 학번은 평점 기준이 없음</t>
         </is>
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아주대학교 전과 안내</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>(학칙 제31조③)</t>
+          <t>신청 자격 · https://www.ajou.ac.kr/kr/bachelor/regs-change.do</t>
         </is>
       </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t>기준 평점을 지어내면 오답</t>
+          <t>학번별로 다르다는 점을 말하면 정답. 모든 학생에게 '평점 2.5 이상'이라고 단정하면 오답</t>
         </is>
       </c>
       <c r="J27" s="10" t="n"/>
@@ -2033,7 +2033,7 @@
       <c r="L27" s="11" t="n"/>
       <c r="M27" s="11" t="inlineStr">
         <is>
-          <t>구간 C · 학사지원 전과 페이지가 DB에 들어오면 정답이 생길 수 있음</t>
+          <t>구간 B · 10/27 재점검: 전과 안내 페이지 추가로 근거 생김 (함정 → B)</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
-          <t>학사지원 휴/복학 안내</t>
+          <t>아주대학교 휴/복학 안내</t>
         </is>
       </c>
       <c r="H41" s="11" t="inlineStr">
@@ -2775,7 +2775,7 @@
       <c r="L41" s="11" t="n"/>
       <c r="M41" s="11" t="inlineStr">
         <is>
-          <t>구간 A · 근거 페이지가 DB에 들어오기 전에는 오답 예상</t>
+          <t>구간 A · 10/25 이전 DB에는 근거 없음 → RAG 전후 비교 사례</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2810,7 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>학사지원 휴/복학 안내</t>
+          <t>아주대학교 휴/복학 안내</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -2828,7 +2828,7 @@
       <c r="L42" s="11" t="n"/>
       <c r="M42" s="11" t="inlineStr">
         <is>
-          <t>구간 A · 근거 페이지가 DB에 들어오기 전에는 오답 예상</t>
+          <t>구간 A · 10/25 이전 DB에는 근거 없음 → RAG 전후 비교 사례</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="G43" s="11" t="inlineStr">
         <is>
-          <t>학사지원 휴/복학 안내</t>
+          <t>아주대학교 휴/복학 안내</t>
         </is>
       </c>
       <c r="H43" s="11" t="inlineStr">
@@ -2881,7 +2881,7 @@
       <c r="L43" s="11" t="n"/>
       <c r="M43" s="11" t="inlineStr">
         <is>
-          <t>구간 A · 근거 페이지가 DB에 들어오기 전에는 오답 예상</t>
+          <t>구간 A · 10/25 이전 DB에는 근거 없음 → RAG 전후 비교 사례</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2916,7 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>학사지원 휴/복학 안내</t>
+          <t>아주대학교 휴/복학 안내</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -2934,7 +2934,7 @@
       <c r="L44" s="11" t="n"/>
       <c r="M44" s="11" t="inlineStr">
         <is>
-          <t>구간 A · 근거 페이지가 DB에 들어오기 전에는 오답 예상</t>
+          <t>구간 A · 10/25 이전 DB에는 근거 없음 → RAG 전후 비교 사례</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="G45" s="11" t="inlineStr">
         <is>
-          <t>학사지원 휴/복학 안내</t>
+          <t>아주대학교 휴/복학 안내</t>
         </is>
       </c>
       <c r="H45" s="11" t="inlineStr">
@@ -2987,7 +2987,7 @@
       <c r="L45" s="11" t="n"/>
       <c r="M45" s="11" t="inlineStr">
         <is>
-          <t>구간 A · 근거 페이지가 DB에 들어오기 전에는 오답 예상</t>
+          <t>구간 A · 10/25 이전 DB에는 근거 없음 → RAG 전후 비교 사례</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>학부 절차를 맞게 말하면 정답</t>
+          <t>학부 절차(보증인 연서·학과장 확인 → 자퇴원서 → 총장 허가)나 학사서비스 자퇴신청 메뉴를 맞게 안내하면 정답</t>
         </is>
       </c>
       <c r="J46" s="10" t="n"/>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>함정-무근거</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
@@ -3176,22 +3176,22 @@
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>(자료에 없음 → 안내가 정답)</t>
+          <t>포털(AIMS2) → 주요서비스 → 증명서발급에서 인터넷 즉시 발급(24시간), 또는 종합지원센터(신학생회관 116호) 앞 무인증명발급기</t>
         </is>
       </c>
       <c r="G49" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아주대학교 증명서 발급 안내</t>
         </is>
       </c>
       <c r="H49" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>인터넷증명서 즉시 발급, 무인증명서 발급기 · https://www.ajou.ac.kr/kr/life/paper01.do</t>
         </is>
       </c>
       <c r="I49" s="11" t="inlineStr">
         <is>
-          <t>발급 방법을 지어내면 오답</t>
+          <t>인터넷 발급이나 무인발급기 중 하나 이상 맞게 안내하면 정답</t>
         </is>
       </c>
       <c r="J49" s="10" t="n"/>
@@ -3199,7 +3199,7 @@
       <c r="L49" s="11" t="n"/>
       <c r="M49" s="11" t="inlineStr">
         <is>
-          <t>구간 C</t>
+          <t>구간 A · 10/27 재점검: 증명서 발급 안내 페이지 추가로 근거 생김 (함정 → A)</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>함정-무근거</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
@@ -3282,22 +3282,22 @@
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>(학사일정 7건에 없음 → 안내가 정답)</t>
+          <t>2학기 수강 정정은 9월 초 (정확한 날짜는 매 학기 공지)</t>
         </is>
       </c>
       <c r="G51" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아주대학교 수강신청 안내</t>
         </is>
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>수강신청 일정 · https://www.ajou.ac.kr/kr/bachelor/enrolment.do</t>
         </is>
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>날짜를 지어내면 오답</t>
+          <t>9월 초를 말하면 정답. 구체 날짜를 지어내면 오답</t>
         </is>
       </c>
       <c r="J51" s="10" t="n"/>
@@ -3305,7 +3305,7 @@
       <c r="L51" s="11" t="n"/>
       <c r="M51" s="11" t="inlineStr">
         <is>
-          <t>구간 C · 학사일정 전체가 수집되면 정답이 생길 수 있음</t>
+          <t>구간 A · 10/27 재점검: 수강신청 안내 페이지 추가로 근거 생김 (함정 → A)</t>
         </is>
       </c>
     </row>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>금액을 지어내면 오답</t>
+          <t>금액을 지어내거나 유학생 학비(₩4,916,000)를 국내생 등록금처럼 말하면 오답. 포털 고지서 확인이나 재무회계팀 안내면 정답</t>
         </is>
       </c>
       <c r="J52" s="10" t="n"/>
@@ -3585,37 +3585,37 @@
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>함정-무근거</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>교류학생이 뭐야?</t>
+          <t>외국인 학생 입국할 때 공항 픽업 서비스 있어?</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>What is an exchange student?</t>
+          <t>Is there an airport pickup service for international students when they arrive?</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr">
         <is>
-          <t>외국 대학·기관과의 협약에 따라 본교에서 공부하는 외국인 학생</t>
+          <t>(자료에 없음 → 국제협력처 유학생입학팀 안내가 정답)</t>
         </is>
       </c>
       <c r="G57" s="11" t="inlineStr">
         <is>
-          <t>외국인학생 지원 및 관리에 관한 규칙</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>제2조(용어의 정의) 3호 · https://rules.ajou.ac.kr/IRS/rule/detail/293</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I57" s="11" t="inlineStr">
         <is>
-          <t>"협약에 따라 수학"이 들어가면 정답</t>
+          <t>있다/없다를 지어내면 오답. 유학생입학팀 문의 안내면 정답</t>
         </is>
       </c>
       <c r="J57" s="10" t="n"/>
@@ -3623,7 +3623,7 @@
       <c r="L57" s="11" t="n"/>
       <c r="M57" s="11" t="inlineStr">
         <is>
-          <t>구간 A</t>
+          <t>구간 C · 10/27 재점검: 기존 '교류학생이 뭐야?'(용어 정의)를 새 함정으로 교체</t>
         </is>
       </c>
     </row>
@@ -3933,7 +3933,7 @@
       </c>
       <c r="I63" s="11" t="inlineStr">
         <is>
-          <t>대학일자리플러스센터가 들어가면 정답</t>
+          <t>대학일자리플러스센터나 유학생입학팀 취업특강을 안내하면 정답</t>
         </is>
       </c>
       <c r="J63" s="10" t="n"/>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="G70" s="11" t="inlineStr">
         <is>
-          <t>학사지원 졸업 안내</t>
+          <t>아주대학교 졸업 안내</t>
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr">
@@ -4312,7 +4312,7 @@
       <c r="L70" s="11" t="n"/>
       <c r="M70" s="11" t="inlineStr">
         <is>
-          <t>구간 A · 근거 페이지가 DB에 들어오기 전에는 오답 예상</t>
+          <t>구간 A · 10/25 이전 DB에는 근거 없음 → RAG 전후 비교 사례</t>
         </is>
       </c>
     </row>
@@ -4486,7 +4486,7 @@
       </c>
       <c r="C74" s="12" t="inlineStr">
         <is>
-          <t>함정-무근거</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
@@ -4501,22 +4501,22 @@
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
-          <t>(체류관리 세부 기준은 자료에 없음 → 국제협력처 유학생입학팀 안내가 정답)</t>
+          <t>체류기한 만료 전에 관할 출입국관리사무소에서 연장. 서류: 여권·외국인등록증, 체류기간연장신청서, 학비납입증명서, 재학증명서(출석률 표시), 거주확인증 또는 임차계약서, 수수료 60,000원</t>
         </is>
       </c>
       <c r="G74" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아주대학교 비자·체류 안내</t>
         </is>
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
-          <t>(외국인학생 규칙 제5조③: 별도 기준)</t>
+          <t>체류기간 연장 · https://www.ajou.ac.kr/iadmissions/life/visa.do</t>
         </is>
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>절차·서류를 지어내면 오답. 담당 부서 안내면 정답</t>
+          <t>만료 전 출입국관리사무소 신청과 주요 서류를 말하면 정답. 절차·비용을 지어내면 오답</t>
         </is>
       </c>
       <c r="J74" s="10" t="n"/>
@@ -4524,7 +4524,7 @@
       <c r="L74" s="11" t="n"/>
       <c r="M74" s="11" t="inlineStr">
         <is>
-          <t>구간 C</t>
+          <t>구간 A · 10/27 재점검: 비자·체류 안내 페이지 추가로 근거 생김 (함정 → A)</t>
         </is>
       </c>
     </row>
@@ -4569,7 +4569,7 @@
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
-          <t>시간을 지어내면 오답</t>
+          <t>시간을 지어내면 오답. 시간제취업 허가 절차(유학생 담당자 확인 → 출입국 신고) 안내는 정답</t>
         </is>
       </c>
       <c r="J75" s="10" t="n"/>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="C76" s="12" t="inlineStr">
         <is>
-          <t>함정-무근거</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
@@ -4607,22 +4607,22 @@
       </c>
       <c r="F76" s="11" t="inlineStr">
         <is>
-          <t>(자료에 없음 → 생활관 안내가 정답)</t>
+          <t>학기당 ₩747,000~₩1,440,000 (유학생 학비·생활비 안내 기준)</t>
         </is>
       </c>
       <c r="G76" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아주대학교 유학생 학비·생활비 안내</t>
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>기숙사비 · https://www.ajou.ac.kr/iadmissions/undergraduate/tuition.do</t>
         </is>
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>금액을 지어내면 오답</t>
+          <t>금액 범위가 맞으면 정답</t>
         </is>
       </c>
       <c r="J76" s="10" t="n"/>
@@ -4630,7 +4630,7 @@
       <c r="L76" s="11" t="n"/>
       <c r="M76" s="11" t="inlineStr">
         <is>
-          <t>구간 C</t>
+          <t>구간 A · 10/27 재점검: 유학생 학비·생활비 페이지 추가로 근거 생김 (함정 → A)</t>
         </is>
       </c>
     </row>
@@ -5811,7 +5811,7 @@
       </c>
       <c r="C99" s="12" t="inlineStr">
         <is>
-          <t>함정-무근거</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
@@ -5826,22 +5826,22 @@
       </c>
       <c r="F99" s="11" t="inlineStr">
         <is>
-          <t>(자료에 없음 → 기숙사 관련 부서 안내가 정답)</t>
+          <t>세탁실은 각 관과 식당동 지하 1층에 있음</t>
         </is>
       </c>
       <c r="G99" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아주대학교 기숙사(유학생) 안내</t>
         </is>
       </c>
       <c r="H99" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>복지시설 · https://www.ajou.ac.kr/iadmissions/life/dorm.do</t>
         </is>
       </c>
       <c r="I99" s="11" t="inlineStr">
         <is>
-          <t>층수를 지어내면 오답</t>
+          <t>각 관(건물)마다 있고 식당동 지하 1층이라고 하면 정답. 층수를 지어내면 오답</t>
         </is>
       </c>
       <c r="J99" s="10" t="n"/>
@@ -5849,7 +5849,7 @@
       <c r="L99" s="11" t="n"/>
       <c r="M99" s="11" t="inlineStr">
         <is>
-          <t>구간 C · 스모크 C1 시드</t>
+          <t>구간 A · 10/27 재점검: 기숙사(유학생) 안내 페이지 추가로 근거 생김 (함정 → A)</t>
         </is>
       </c>
     </row>

</xml_diff>